<commit_message>
Proceso y de las nuevas implementacions - categorías
</commit_message>
<xml_diff>
--- a/apps/web/public/plantilla_carga_masiva.xlsx
+++ b/apps/web/public/plantilla_carga_masiva.xlsx
@@ -417,17 +417,17 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="str">
-        <v>⚠️ INSTRUCCIONES PARA LA CARGA MASIVA</v>
+        <v>⚠️ PLANTILLA DE CARGA MASIVA - BODEGIA</v>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1">
       <c r="A2" t="str">
-        <v>CAMPOS OBLIGATORIOS (con *): NOMBRE, CÓDIGO, PRECIO COSTO y PRECIO VENTA. Los demás campos son opcionales.</v>
+        <v>Solo son OBLIGATORIOS (*): NOMBRE, CÓDIGO, PRECIO COSTO y PRECIO VENTA. Los demás campos son OPCIONALES.</v>
       </c>
     </row>
     <row r="3" ht="35" customHeight="1">
       <c r="A3" t="str">
-        <v>Si no llenas CATEGORÍA se usará "general", STOCK INICIAL será 0, ESTADO será "Disponible" y STOCK BAJO será 20.</v>
+        <v>Si no llenas: CATEGORÍA=general, STOCK=0, ESTADO=Disponible, STOCK BAJO=20</v>
       </c>
     </row>
     <row r="4" ht="5" customHeight="1"/>
@@ -489,7 +489,7 @@
         <v>6.5</v>
       </c>
       <c r="E6" t="str">
-        <v>comestibles</v>
+        <v>abarrotes</v>
       </c>
       <c r="F6">
         <v>30</v>
@@ -498,7 +498,7 @@
         <v>Disponible</v>
       </c>
       <c r="H6" t="str">
-        <v>10/12/2026</v>
+        <v>2026-12-10</v>
       </c>
       <c r="I6" t="str">
         <v>Primor</v>
@@ -513,10 +513,10 @@
         <v>20123456789</v>
       </c>
       <c r="M6" t="str">
-        <v>http://imagen.com/aceite.jpg</v>
+        <v/>
       </c>
       <c r="N6">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>